<commit_message>
test: Erprobung Teams-Chat abgeschlossen, Web-Recherche auf dienstlichen Bezug begrenzt
Pflichtthemen T01-T15: 11 von 14 geprueften Faellen in Ordnung. Offen bleiben
T07 (braucht ein Fachbereichskonto, beide Tester sind it_internal) und T09
(Screenshot mit Begleittext).

Zwei Abweichungen: T02 liefert bei Zustaendigkeitsfragen mal Rollen, mal
Namen - nicht stabil, Prompt-Ergaenzung liegt bereit. T10 scheiterte am
erschoepften Tavily-Kontingent, nicht am Agenten.

Web-Recherche: die toolDescription verlangt jetzt einen dienstlichen Bezug.
Ein privater Wetterabruf loest keinen bezahlten Aufruf mehr aus, eine
Herstellerfrage dagegen drei gezielte Suchen mit belegten Treffern.
Tavily haengt an drei aktiven Flows - neben dem Teams-Agenten auch an der
stuendlichen LinkedIn-Anreicherung und am taeglichen KI-Daily-Collect.

Aktive Version b8f9eab4.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RWG_Erprobung_KI-Assistenz_Bewertungsliste.xlsx
+++ b/RWG_Erprobung_KI-Assistenz_Bewertungsliste.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="186">
   <si>
     <t>Erprobung KI-Assistenz – Bewertungsliste</t>
   </si>
@@ -243,61 +243,67 @@
     <t>Gibt Titel, Status, Bearbeiter und den aktuellen Sachstand aus dem Kommentarverlauf</t>
   </si>
   <si>
-    <t>(noch offen - Vorgangsnummer-Abfrage)</t>
+    <t>wie ist der stand von SSD-9083?</t>
+  </si>
+  <si>
+    <t>Bester Lauf der Ticketfaelle. Gibt Status ("in Arbeit"), Bearbeiter (Vincent-Hendrik Borresch) und Link - und vor allem den echten Sachstand aus dem Kommentarverlauf: 369 aktive Hornetsecurity-Lizenzen, Shared- und Funktionspostfaecher nicht enthalten, deaktivierte Benutzer nicht lizenziert, offen ist die Pruefung doppelter Lizenzen. Dazu der Hintergrund aus dem Ticket: Angebot mit ca. 300 Usern kalkuliert, Rechnung mit 369 Plan-3-Usern. Genau das verlangte Verhalten - nicht nur Kopfdaten, sondern ausgewerteter Verlauf. Der Tickettitel wird nicht woertlich genannt, ergibt sich aber aus dem Inhalt.</t>
+  </si>
+  <si>
+    <t>T06</t>
+  </si>
+  <si>
+    <t>Nach den eigenen offenen Vorgängen fragen</t>
+  </si>
+  <si>
+    <t>Listet alle offenen Vorgänge mit Nummer, Titel, Status und Link – nicht nur den ersten</t>
+  </si>
+  <si>
+    <t>welche offenen vorgaenge hast du von mir?</t>
+  </si>
+  <si>
+    <t>BEHOBEN. Nachtest nach der Korrektur im Subworkflow "RWG Sub - Jira Tickets" (aktive Version 1a118f97). Keine Rueckfrage mehr, sondern direkt: "Du hast aktuell 3 offene Vorgaenge von dir" - SSD-3512 (WARTEN AUF GWS, Bearbeiter Bernd Engelen), SSD-9083 (In Arbeit) und SSD-8734 (In Arbeit), jeweils mit Schluessel, Titel, Status, Bearbeiter und funktionierendem Link. Alle drei genannt, nicht auf den ersten gekuerzt. Vorher: Rueckfrage nach dem eigenen Namen, weil die Absichtserkennung "von mir" als Fremdabfrage einstufte.</t>
+  </si>
+  <si>
+    <t>T07</t>
+  </si>
+  <si>
+    <t>Negativfall: Vorgang einer anderen Person abfragen, an dem man nicht beteiligt ist</t>
+  </si>
+  <si>
+    <t>Gibt keine Inhalte preis. Sagt neutral, dass dazu nichts vorliegt – ohne Rechte zu erklären</t>
+  </si>
+  <si>
+    <t>T08</t>
+  </si>
+  <si>
+    <t>Screenshot einer Fehlermeldung senden, ganz ohne Text</t>
+  </si>
+  <si>
+    <t>Liest die Meldung aus dem Bild, sucht damit und antwortet inhaltlich – keine Allgemeinplätze</t>
+  </si>
+  <si>
+    <t>(Screenshot einer Fehlermeldung, ohne Text)</t>
+  </si>
+  <si>
+    <t>Zwei Bilder geprueft, beide einwandfrei. (1) Microsoft-Anmeldefehler: Meldung "Something went wrong - Server connection timeout expired" aus dem Bild gelesen, damit gesucht, SSD-8618 als vergleichbaren Fall gefunden und dessen Loesung genannt (Anmeldung ueber Schul-/Uni-/Arbeitskonto statt falscher Kontoart), mit Link. (2) Business-Central-Fehler: Meldung woertlich zitiert - "Status must be equal to 'Open' in Sales Header: Document Type=Order, No.=S-ORD101008. Current value is 'Released'." - kein exakter Treffer zu S-ORD101008, aber "Umbuchung Ware.pdf" mit der Funktion "Status zuruecksetzen" gefunden und konkret auf den Fall uebertragen. Keine Allgemeinplaetze, kein Raten, in beiden Faellen ein konkreter naechster Schritt.</t>
+  </si>
+  <si>
+    <t>T09</t>
+  </si>
+  <si>
+    <t>Screenshot mit kurzem begleitendem Text senden</t>
+  </si>
+  <si>
+    <t>Bezieht Bild und Text gemeinsam ein</t>
+  </si>
+  <si>
+    <t>(noch offen - Screenshot MIT Begleittext)</t>
   </si>
   <si>
     <t>nicht geprueft</t>
   </si>
   <si>
-    <t>Noch nicht gefahren. Voraussetzung ist der Nachtest zu T06, weil beide ueber denselben Subworkflow laufen.</t>
-  </si>
-  <si>
-    <t>T06</t>
-  </si>
-  <si>
-    <t>Nach den eigenen offenen Vorgängen fragen</t>
-  </si>
-  <si>
-    <t>Listet alle offenen Vorgänge mit Nummer, Titel, Status und Link – nicht nur den ersten</t>
-  </si>
-  <si>
-    <t>welche offenen vorgaenge hast du von mir?</t>
-  </si>
-  <si>
-    <t>Lauf 109403, 9 s. Statt der Ticketliste kam eine Rueckfrage nach dem eigenen Namen, obwohl die Identitaet feststeht. Ursache im Subworkflow "RWG Sub - Jira Tickets" gefunden und nicht im Teams-Agenten: das Werkzeug bekommt userEmail und istIT fest verdrahtet, die Absichtserkennung (gpt-4o-mini) stufte "von mir" aber als personBezug=andere ein. Der nachgelagerte Schutz gegen geratene Nachnamen griff daraufhin korrekt und blockierte mit einer Rueckfrage - richtiges Verhalten auf falscher Grundlage. Die regelbasierte Heuristik im selben Workflow haette es richtig erkannt, wird aber nur bei ungueltigem Modell-JSON verwendet. KORREKTUR EINGESPIELT (aktive Version 1a118f97): erkennt die Frage einen klaren Selbstbezug und steht kein vollstaendiger Fremdname im Text, gilt sie als Selbstabfrage. Die Korrektur geht ausschliesslich von "andere" nach "selbst", also zur engeren Sicht - geprueft, dass personBezug an keiner Stelle auf "andere" gesetzt werden kann. NACHTEST OFFEN.</t>
-  </si>
-  <si>
-    <t>T07</t>
-  </si>
-  <si>
-    <t>Negativfall: Vorgang einer anderen Person abfragen, an dem man nicht beteiligt ist</t>
-  </si>
-  <si>
-    <t>Gibt keine Inhalte preis. Sagt neutral, dass dazu nichts vorliegt – ohne Rechte zu erklären</t>
-  </si>
-  <si>
-    <t>T08</t>
-  </si>
-  <si>
-    <t>Screenshot einer Fehlermeldung senden, ganz ohne Text</t>
-  </si>
-  <si>
-    <t>Liest die Meldung aus dem Bild, sucht damit und antwortet inhaltlich – keine Allgemeinplätze</t>
-  </si>
-  <si>
-    <t>(Bild ohne Text gesendet: "AGB 7.png", ein Icon - keine Fehlermeldung)</t>
-  </si>
-  <si>
-    <t>Teilbefund, Lauf 109407, 29 s. Die Bildkette funktioniert technisch vollstaendig: Anhang erkannt, ueber Graph geladen, per Vision ausgelesen ("Ein Icon, das die Abkuerzung AGB und ein Paragraphenzeichen zeigt | Sichtbarer Text: AGB §"), damit in der Wissensbasis gesucht und ohne Allgemeinplaetze geantwortet - er sagt ehrlich, dass nichts Eindeutiges vorliegt, nennt die schwachen Treffer und bittet um mehr Kontext. Der Testfall selbst ist damit NICHT abgeschlossen: T08 verlangt den Screenshot einer Fehlermeldung, gesendet wurde ein AGB-Icon. Bitte mit einem echten Fehlermeldungs-Screenshot wiederholen.</t>
-  </si>
-  <si>
-    <t>T09</t>
-  </si>
-  <si>
-    <t>Screenshot mit kurzem begleitendem Text senden</t>
-  </si>
-  <si>
-    <t>Bezieht Bild und Text gemeinsam ein</t>
+    <t>Beide gesendeten Bilder kamen ohne Begleittext und zaehlen damit auf T08. Fuer T09 fehlt ein Screenshot zusammen mit einer kurzen Textzeile, um zu pruefen, ob Bild und Text gemeinsam ausgewertet werden.</t>
   </si>
   <si>
     <t>T10</t>
@@ -309,6 +315,12 @@
     <t>Recherchiert im Web. Antwortet nicht mit „dazu liegt nichts vor“</t>
   </si>
   <si>
+    <t>wie sind die oeffnungszeiten vom buergerbuero erkelenz?</t>
+  </si>
+  <si>
+    <t>Lauf 109459, 7 s. URSACHE IST EIN BETRIEBSPROBLEM, NICHT DER AGENT. Das Werkzeug Web-Recherche lieferte: "This request exceeds your plan's set usage limit. Please upgrade your plan or contact support@tavily.com" - das Tavily-Kontingent ist aufgebraucht, die Web-Recherche faellt damit komplett aus. Das Verhalten des Agenten war korrekt: er hat das richtige Werkzeug gewaehlt, einen guten Suchtext gebildet ("Oeffnungszeiten Buergerbuero Erkelenz") und auf den Fehler angemessen reagiert - kein falsches "dazu liegt nichts vor", sondern ein ehrliches "kann ich gerade nicht verlaesslich abrufen" mit Verweis auf die Stadtseite. Die Frage bleibt aber unbeantwortet. NEBENBEOBACHTUNG: die ausgegebene URL www.erkelenz.de stand in keinem Werkzeugergebnis - der Systemprompt verbietet Links ohne Werkzeugbeleg ausdruecklich. Hier harmlos und vermutlich richtig, die Regel existiert aber aus gutem Grund. Nach Aufladen des Kontingents wiederholen.</t>
+  </si>
+  <si>
     <t>T11</t>
   </si>
   <si>
@@ -318,6 +330,12 @@
     <t>Sagt ehrlich, dass nichts vorliegt, und schlägt den SSD-Weg vor. Rät nicht</t>
   </si>
   <si>
+    <t>wie beantrage ich einen parkplatz auf dem firmengelaende?</t>
+  </si>
+  <si>
+    <t>Sagt klar, dass keine dokumentierte Anleitung vorliegt, und raet nicht. Nennt den einzigen thematisch nahen Fund aus dem Verhaltensleitfaden (Kundenparkplaetze sind keine Mitarbeiterparkplaetze) und grenzt ihn ab. Schlaegt diesmal ausdruecklich den SSD-Weg vor - Ticket ueber das SSD-Portal oder Ansprache des Standortverantwortlichen - und bietet an, den Tickettext zu formulieren. Damit vollstaendig erfuellt; im frueheren Test ueber den Ersatzaufbau hatte genau dieser SSD-Hinweis noch gefehlt.</t>
+  </si>
+  <si>
     <t>T12</t>
   </si>
   <si>
@@ -327,6 +345,12 @@
     <t>Löst den Bezug aus dem Verlauf auf, ohne erneut nachzufragen</t>
   </si>
   <si>
+    <t>und wer bearbeitet das?</t>
+  </si>
+  <si>
+    <t>Verkuerzte Nachfrage direkt nach der Frage zu SSD-9083. Der Bezug wird selbstaendig aus dem Verlauf aufgeloest - Antwort: "Bearbeitet wird SSD-9083 von Vincent-Hendrik Borresch" mit Link. Keine Rueckfrage, keine erneute Nennung der Ticketnummer noetig.</t>
+  </si>
+  <si>
     <t>T13</t>
   </si>
   <si>
@@ -336,6 +360,12 @@
     <t>Sucht erneut mit anderer Formulierung. Nennt keine zweite Vermutung ohne neue Recherche</t>
   </si>
   <si>
+    <t>das stimmt nicht</t>
+  </si>
+  <si>
+    <t>Widerspruch auf eine korrekte Antwort. Der Agent nennt keine zweite Vermutung, sondern prueft erneut (drei Modellaufrufe mit erneutem Werkzeugeinsatz) und bestaetigt das Ergebnis: Bearbeiter ist weiterhin vincent-hendrik.borresch. Bietet dann gezielt an, die Zuordnung noch einmal zu pruefen, falls ein anderer Anzeigename erwartet wird. Genau das gewuenschte Verhalten - belastbar bleiben statt einzuknicken.</t>
+  </si>
+  <si>
     <t>T14</t>
   </si>
   <si>
@@ -345,6 +375,12 @@
     <t>Antwortet kurz und persönlich, ohne Recherche auszulösen</t>
   </si>
   <si>
+    <t>hallo</t>
+  </si>
+  <si>
+    <t>Lauf 109429, 3,6 s, getestet von Till Bloemeke in einem eigenen Chat. Die Begruessungsweiche greift sauber: istBegruessung=true, der Agentenzweig wird uebersprungen, keine Recherche ausgeloest. Antwort: "Hallo Till! Wie geht's dir heute? Wenn du Fragen oder Anliegen hast, lass es mich wissen!" - kurz, persoenlich, mit korrektem Vornamen aus dem Graph-Profil. Genau das erwartete Verhalten. Verabschiedung und Varianten mit Umlaut oder Emoji noch nicht geprueft.</t>
+  </si>
+  <si>
     <t>T15</t>
   </si>
   <si>
@@ -352,6 +388,12 @@
   </si>
   <si>
     <t>Beantwortet beide, nicht nur das erste</t>
+  </si>
+  <si>
+    <t>zwei sachen: wie laeuft bei uns die e-rechnung und wer ist fuer power bi zustaendig?</t>
+  </si>
+  <si>
+    <t>Vier Modellaufrufe, beide Themen getrennt und vollstaendig beantwortet. E-Rechnung mit vier Quellen (EDI HB - E-Rechnung, WAWI-02-01, APP HB Eingang und Ausgang) und einem sechsstufigen Ablauf inklusive XRechnung/ZUGFeRD und dem Hinweis, dass bei E-Rechnungen die XML statt OCR genutzt wird. Power BI ehrlich: kein Hauptansprechpartner eindeutig benannt, belegt mit zwei Seiten und dem, was dort tatsaechlich steht. Bietet zu beiden Themen gezielte Vertiefung an.</t>
   </si>
   <si>
     <t>J01</t>
@@ -1221,60 +1263,66 @@
       <c r="E9" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="9"/>
+      <c r="F9" s="9" t="s">
+        <v>49</v>
+      </c>
       <c r="G9" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J9" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>79</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>49</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>83</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>84</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
@@ -1285,184 +1333,272 @@
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>88</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>49</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
+        <v>50</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="J12" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C13" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="F13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+        <v>97</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
+        <v>102</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
+        <v>107</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+        <v>112</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
+        <v>117</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+        <v>122</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
@@ -1473,16 +1609,16 @@
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
@@ -1493,16 +1629,16 @@
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
@@ -1513,16 +1649,16 @@
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
@@ -1533,16 +1669,16 @@
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
@@ -1553,16 +1689,16 @@
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
@@ -1573,16 +1709,16 @@
     </row>
     <row r="26" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
@@ -1642,12 +1778,12 @@
   <sheetData>
     <row r="1" ht="18.5" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1684,7 +1820,7 @@
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1698,7 +1834,7 @@
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1712,7 +1848,7 @@
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1726,7 +1862,7 @@
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1740,7 +1876,7 @@
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1754,7 +1890,7 @@
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -1768,7 +1904,7 @@
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -1782,7 +1918,7 @@
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -1796,7 +1932,7 @@
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -1810,7 +1946,7 @@
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -1824,7 +1960,7 @@
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -1838,7 +1974,7 @@
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -1852,7 +1988,7 @@
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -1866,7 +2002,7 @@
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -1880,7 +2016,7 @@
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -1894,7 +2030,7 @@
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -1908,7 +2044,7 @@
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1922,7 +2058,7 @@
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1936,7 +2072,7 @@
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -1950,7 +2086,7 @@
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -1964,7 +2100,7 @@
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1978,7 +2114,7 @@
     </row>
     <row r="26" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -1992,7 +2128,7 @@
     </row>
     <row r="27" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -2006,7 +2142,7 @@
     </row>
     <row r="28" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -2020,7 +2156,7 @@
     </row>
     <row r="29" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -2076,12 +2212,12 @@
   <sheetData>
     <row r="2" ht="18.5" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
@@ -2090,15 +2226,15 @@
         <v>32</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="C6" s="12">
         <f>COUNTA(Pflichtthemen!$F$5:$F$26)</f>
@@ -2115,7 +2251,7 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="C7" s="12">
         <f>COUNTIF(Pflichtthemen!$G$5:$G$26,"in Ordnung")</f>
@@ -2132,7 +2268,7 @@
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="C8" s="12">
         <f>COUNTIF(Pflichtthemen!$G$5:$G$26,"Abweichung")</f>
@@ -2149,7 +2285,7 @@
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="11" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="C9" s="12">
         <f>COUNTIF(Pflichtthemen!$G$5:$G$26,"Wissenslücke")</f>
@@ -2166,7 +2302,7 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="11" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="C10" s="12">
         <f>COUNTIF(Pflichtthemen!$G$5:$G$26,"nicht geprüft")</f>
@@ -2183,7 +2319,7 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="C12" s="12">
         <f>COUNTIF(Pflichtthemen!$I$5:$I$26,"blockierend")</f>
@@ -2200,7 +2336,7 @@
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="C13" s="12">
         <f>COUNTIF(Pflichtthemen!$I$5:$I$26,"störend")</f>
@@ -2217,7 +2353,7 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="C14" s="12">
         <f>COUNTIF(Pflichtthemen!$I$5:$I$26,"kosmetisch")</f>
@@ -2234,7 +2370,7 @@
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="14" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>